<commit_message>
small adjustment in the 'Object__to_from_node' so the connection value is as user defined RES capacity
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/methane/Model_Data_Base_methane_updated.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/methane/Model_Data_Base_methane_updated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kar.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\methane\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D4CD41-9B31-4A11-BB41-1F93B743D2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF09A765-5BD1-4CE1-AB77-64803296BCDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="4575" yWindow="4290" windowWidth="38700" windowHeight="15345" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -1371,7 +1371,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C870BDA0-9E4C-481D-87BE-9D47789809C8}">
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -1397,7 +1397,7 @@
     <col min="26" max="26" width="37.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1477,7 +1477,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>65</v>
       </c>
@@ -1536,7 +1536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>66</v>
       </c>
@@ -1592,7 +1592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>67</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>68</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>110</v>
       </c>
@@ -1715,15 +1715,14 @@
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7"/>
-      <c r="Y6" s="7"/>
-      <c r="Z6" s="7" t="s">
+      <c r="Y6" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="AA6" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z6" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>112</v>
       </c>
@@ -1768,15 +1767,14 @@
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
       <c r="X7" s="4"/>
-      <c r="Y7" s="4"/>
-      <c r="Z7" s="4" t="s">
+      <c r="Y7" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AA7" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z7" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>113</v>
       </c>
@@ -1835,15 +1833,14 @@
       <c r="V8" s="7"/>
       <c r="W8" s="7"/>
       <c r="X8" s="7"/>
-      <c r="Y8" s="7"/>
-      <c r="Z8" s="7" t="s">
+      <c r="Y8" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="AA8" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z8" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>115</v>
       </c>
@@ -1888,15 +1885,14 @@
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
       <c r="X9" s="4"/>
-      <c r="Y9" s="4"/>
-      <c r="Z9" s="4" t="s">
+      <c r="Y9" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AA9" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z9" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>116</v>
       </c>
@@ -1955,15 +1951,14 @@
       <c r="V10" s="7"/>
       <c r="W10" s="7"/>
       <c r="X10" s="7"/>
-      <c r="Y10" s="7"/>
-      <c r="Z10" s="7" t="s">
+      <c r="Y10" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="AA10" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z10" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>118</v>
       </c>
@@ -2008,11 +2003,10 @@
       <c r="V11" s="4"/>
       <c r="W11" s="4"/>
       <c r="X11" s="4"/>
-      <c r="Y11" s="4"/>
-      <c r="Z11" s="4" t="s">
+      <c r="Y11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AA11" s="10">
+      <c r="Z11" s="10">
         <v>1</v>
       </c>
     </row>

</xml_diff>